<commit_message>
Rebuild Quan_ly_cho_vay workbook with visible TC mới sheet
Ensure sheet TC mới is first/active in the output Excel named
like the user file so the new cases are immediately visible.

Co-authored-by: Nguyen-Ha123 <Nguyen-Ha123@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Quan_ly_cho_vay_ fix comment.xlsx
+++ b/output/Quan_ly_cho_vay_ fix comment.xlsx
@@ -101,12 +101,6 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -114,6 +108,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -499,374 +499,374 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID_UC</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ID_TC</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tiêu đề</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Tiền điều kiện</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Các bước thực hiện</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Kết quả mong muốn</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Kết quả test</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr"/>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Sửa hồ sơ (Danh sách — sheet đầu)</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>SECTION — TC mới (bôi vàng)</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>SECTION</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_001</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Hiển thị action Sửa trên danh sách hồ sơ</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có ≥1 hồ sơ trên lưới.</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>1. Quan sát cột Thao tác / action trên từng dòng hồ sơ
 2. Hover / kiểm tra icon hoặc nút Sửa</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Mỗi dòng hồ sơ hợp lệ hiển thị action Sửa (icon/bút chì hoặc menu).
 Action nhận diện được, không bị che.</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_002</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Mở form Sửa Hồ sơ - Uỷ thác cho vay từ danh sách</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có ≥1 hồ sơ.</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>1. Tại dòng hồ sơ bất kỳ, click Sửa
 2. Quan sát popup/form mở ra</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Mở form tiêu đề: "Sửa Hồ sơ - Uỷ thác cho vay".
 Có nút đóng (X), Hủy, Lưu.
 Form load đủ section theo UI (Hình thức tiếp nhận, Người nộp, Thông tin tờ khai, Dự án, Đề nghị vay, Giải ngân, Thẩm định/Tài sản, Hồ sơ đính kèm).</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_003</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Form Sửa prefill đúng dữ liệu hồ sơ đã lưu</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Biết sẵn giá trị các field của 1 hồ sơ (gồm phần tài sản).</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>1. Click Sửa trên hồ sơ đã chọn
 2. So sánh từng field trên form với dữ liệu đã lưu / chi tiết hồ sơ</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Toàn bộ field hiển thị đúng giá trị hiện tại của hồ sơ (không blank sai, không lệch sang hồ sơ khác).
 Gồm cả field tài sản: Tài sản đảm bảo, Mô tả chi tiết TSĐB, Hiện trạng tài sản, Tính pháp lý tài sản.</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_004</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Sửa — Hủy không lưu thay đổi</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Mở form Sửa.</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>1. Đổi giá trị 1 field bất kỳ (vd: Họ tên người nộp)
 2. Click Hủy
 3. Mở lại Sửa / Chi tiết cùng hồ sơ</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Form đóng, không lưu.
 Dữ liệu hồ sơ giữ nguyên giá trị cũ.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_005</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Sửa — đóng icon X không lưu</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Mở form Sửa.</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>1. Đổi 1 field
 2. Click icon X
 3. Kiểm tra lại dữ liệu hồ sơ</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Form đóng, không lưu. Dữ liệu gốc không đổi.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_006</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Sửa — bỏ trống field bắt buộc (Người nộp / Tổ chức)</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Mở form Sửa. Các field (*) đang có giá trị.</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>1. Xóa trống lần lượt các field (*): Loại giấy tờ người nộp / Số định danh / Họ tên người nộp / Mã số thuế / các field (*) khác visible
 2. Click Lưu</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Không lưu thành công.
 Highlight field lỗi + message kiểu "Vui lòng nhập + tên trường" (theo UI thực tế).
 Nút Lưu disabled hoặc form vẫn mở. [TBD message nguyên văn nếu SRS khác]</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Assumption: rule required giống form Tạo mới</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_007</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Sửa phần Tài sản đảm bảo — happy path</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Hồ sơ cho phép sửa. Mở form Sửa → section "5. Kết quả thẩm định hồ sơ của ngân hàng".</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>1. Sửa "Tài sản đảm bảo" = giá trị hợp lệ mới
 2. Sửa "Mô tả chi tiết tài sản đảm bảo"
@@ -877,144 +877,144 @@
 7. Mở Chi tiết / Sửa lại để verify</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Lưu thành công (message theo UI, vd: "Cập nhật thành công" — [TBD]).
 4 field tài sản phản ánh đúng giá trị mới trên Chi tiết hồ sơ.
 Các field khác không bị ghi đè sai.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_008</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Sửa phần Tài sản — bỏ trống field (*) tài sản</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Mở form Sửa, section thẩm định/tài sản.</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>1. Xóa trống lần lượt: Tài sản đảm bảo / Mô tả chi tiết TSĐB / Hiện trạng tài sản / Tính pháp lý tài sản
 2. Click Lưu sau mỗi lần (hoặc cuối cùng)</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Không cho lưu khi field (*) tài sản trống.
 Hiển thị validation + highlight field.
 Message: "Vui lòng nhập + tên trường" (ưu tiên text UI).</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_009</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Sửa — cập nhật Hình thức tiếp nhận (Trực tiếp / Trực tuyến)</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Mở form Sửa.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>1. Đổi radio Hình thức từ Trực tiếp ↔ Trực tuyến
 2. Click Lưu
 3. Mở lại form / chi tiết</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Lưu thành công. Hình thức hiển thị đúng lựa chọn mới.</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr"/>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>TC_EDIT_010</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Sửa — không cho sửa / ẩn Sửa theo trạng thái hồ sơ (nếu có rule)</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có hồ sơ ở các trạng thái: Chờ tiếp nhận, Chờ phân công, Chờ thẩm định, Chờ ký duyệt, Đã ký duyệt.</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>1. Với từng trạng thái, kiểm tra action Sửa trên danh sách
 2. Nếu mở được form: thử Lưu thay đổi nhỏ</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Theo business rule [TBD từ SRS]:
 - Trạng thái cho phép sửa → action Sửa available, lưu OK
@@ -1022,210 +1022,210 @@
 Ghi nhận thực tế UI vào Kết quả test.</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>BLOCKED/TBD — cần confirm rule theo trạng thái từ SRS</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Xóa hồ sơ (Danh sách — sheet đầu)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>SECTION — TC mới (bôi vàng)</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>SECTION</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>TC_DEL_001</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Hiển thị action Xóa trên danh sách hồ sơ</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có ≥1 hồ sơ.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>1. Quan sát cột Thao tác trên lưới
 2. Kiểm tra icon/nút Xóa</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Action Xóa hiển thị trên dòng hồ sơ (theo quyền + trạng thái cho phép).</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>TC_DEL_002</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Xóa hồ sơ — hủy trên dialog xác nhận</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Chọn 1 hồ sơ còn trên list.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>1. Click Xóa
 2. Quan sát dialog xác nhận
 3. Chọn Hủy / Không / Đóng</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Hiện dialog xác nhận xóa (nội dung rõ mã/tên hồ sơ nếu có).
 Sau khi Hủy: dialog đóng, hồ sơ vẫn còn trên danh sách, dữ liệu không đổi.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>TC_DEL_003</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Xóa hồ sơ — xác nhận thành công</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có hồ sơ test chuyên dụng (không ảnh hưởng data thật).</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>1. Ghi nhận mã/ID hồ sơ trước khi xóa
 2. Click Xóa → Xác nhận
 3. Quan sát danh sách + (nếu có) tìm lại theo mã</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Message thành công theo UI (vd: "Xóa thành công" — [TBD]).
 Hồ sơ biến mất khỏi danh sách.
 Search lại mã → Không có dữ liệu / không tìm thấy.</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>TC_DEL_004</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Xóa hồ sơ — ràng buộc theo trạng thái</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có hồ sơ từng trạng thái process (Chờ tiếp nhận … Đã ký duyệt).</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>1. Thử Xóa với từng trạng thái
 2. Ghi nhận cho phép / chặn</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Theo rule [TBD]:
 - Trạng thái cho phép xóa → xóa OK như TC_DEL_003
@@ -1233,119 +1233,119 @@
 Ưu tiên behavior UI thực tế.</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>TBD rule theo trạng thái</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>TC_DEL_005</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Xóa hồ sơ — kiểm tra phần tài sản/thẩm định bị gỡ theo hồ sơ</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Hồ sơ có dữ liệu section tài sản đã lưu; trạng thái cho phép xóa.</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>1. Mở Chi tiết xác nhận có dữ liệu Tài sản đảm bảo / TSĐB
 2. Quay lại danh sách → Xóa → Xác nhận
 3. Cố mở lại chi tiết / query theo ID (nếu có quyền/API/DB)</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Hồ sơ và dữ liệu liên quan (gồm phần tài sản/thẩm định) không còn truy cập được trên UI.
 Không còn orphan hiển thị trên list. [TBD SQL table nếu SRS cung cấp]</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Chi tiết hồ sơ — Thanh process (highlight theo trạng thái)</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>SECTION — TC mới (bôi vàng)</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>SECTION</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_001</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Thanh process hiển thị đủ 5 bước trạng thái</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái tương ứng.</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>1. Mở tab CHI TIẾT HỒ SƠ
 2. Quan sát thanh process phía trên</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Thanh process hiển thị đúng 5 bước theo thứ tự:
 - 1. Chờ tiếp nhận
@@ -1356,92 +1356,92 @@
 Các bước nối nhau trên 1 thanh ngang, nhìn thấy số thứ tự.</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_002</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Highlight process = trạng thái hồ sơ hiện tại (mapping)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái tương ứng. Biết trạng thái hồ sơ trên list / header.</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>1. Đọc trạng thái hồ sơ (list hoặc nhãn trên chi tiết)
 2. So với bước đang được highlight trên thanh process</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Bước được highlight / active trên thanh process KHỚP đúng trạng thái hiện tại của hồ sơ.
 Không highlight sai bước.</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_003</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Process highlight khi trạng thái = Chờ tiếp nhận</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái "Chờ tiếp nhận".</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>1. Mở Chi tiết hồ sơ trạng thái "Chờ tiếp nhận"
 2. Quan sát bước số 1 trên thanh process
 3. Quan sát các bước trước/sau</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Bước 1 "Chờ tiếp nhận" được highlight (active / màu nhấn — theo UI, vd chữ xanh đậm hoặc vòng active).
 Các bước &lt; 1: thể hiện đã qua (completed style).
@@ -1449,47 +1449,47 @@
 Trạng thái hồ sơ = "Chờ tiếp nhận".</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_004</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Process highlight khi trạng thái = Chờ phân công</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái "Chờ phân công".</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>1. Mở Chi tiết hồ sơ trạng thái "Chờ phân công"
 2. Quan sát bước số 2 trên thanh process
 3. Quan sát các bước trước/sau</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Bước 2 "Chờ phân công" được highlight (active / màu nhấn — theo UI, vd chữ xanh đậm hoặc vòng active).
 Các bước &lt; 2: thể hiện đã qua (completed style).
@@ -1497,47 +1497,47 @@
 Trạng thái hồ sơ = "Chờ phân công".</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_005</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Process highlight khi trạng thái = Chờ thẩm định</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái "Chờ thẩm định".</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>1. Mở Chi tiết hồ sơ trạng thái "Chờ thẩm định"
 2. Quan sát bước số 3 trên thanh process
 3. Quan sát các bước trước/sau</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>Bước 3 "Chờ thẩm định" được highlight (active / màu nhấn — theo UI, vd chữ xanh đậm hoặc vòng active).
 Các bước &lt; 3: thể hiện đã qua (completed style).
@@ -1545,47 +1545,47 @@
 Trạng thái hồ sơ = "Chờ thẩm định".</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_006</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Process highlight khi trạng thái = Chờ ký duyệt</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái "Chờ ký duyệt".</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>1. Mở Chi tiết hồ sơ trạng thái "Chờ ký duyệt"
 2. Quan sát bước số 4 trên thanh process
 3. Quan sát các bước trước/sau</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Bước 4 "Chờ ký duyệt" được highlight (active / màu nhấn — theo UI, vd chữ xanh đậm hoặc vòng active).
 Các bước &lt; 4: thể hiện đã qua (completed style).
@@ -1593,47 +1593,47 @@
 Trạng thái hồ sơ = "Chờ ký duyệt".</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_007</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Process highlight khi trạng thái = Đã ký duyệt</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái "Đã ký duyệt".</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>1. Mở Chi tiết hồ sơ trạng thái "Đã ký duyệt"
 2. Quan sát bước số 5 trên thanh process
 3. Quan sát các bước trước/sau</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Bước 5 "Đã ký duyệt" được highlight (active / màu nhấn — theo UI, vd chữ xanh đậm hoặc vòng active).
 Các bước &lt; 5: thể hiện đã qua (completed style).
@@ -1641,132 +1641,132 @@
 Trạng thái hồ sơ = "Đã ký duyệt".</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_008</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Đồng bộ trạng thái List ↔ Process bar Chi tiết</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập hệ thống → vào màn hình Danh sách hồ sơ Uỷ thác cho vay (sheet đầu / danh sách hồ sơ). Có ≥1 hồ sơ mỗi trạng thái (hoặc sample đa trạng thái).</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>1. Từ danh sách, ghi trạng thái cột Trạng thái của hồ sơ A
 2. Click vào hồ sơ A → Chi tiết
 3. Đối chiếu bước highlight trên process bar</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Trạng thái trên list = bước đang highlight trên process bar chi tiết.
 Không lệch (vd list "Chờ thẩm định" mà process highlight "Đã ký duyệt").</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_009</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Thanh process chỉ đọc — không đổi trạng thái bằng click bước</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái tương ứng.</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>1. Click lần lượt các bước trên thanh process
 2. Quan sát trạng thái hồ sơ / highlight</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>Click bước không làm thay đổi trạng thái hồ sơ.
 Highlight vẫn theo trạng thái hiện tại.
 Không có navigation/action ngoài ý muốn (trừ khi SRS định nghĩa — [TBD]).</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_010</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Process bar vẫn hiển thị khi chuyển tab chi tiết</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>Đăng nhập → Danh sách hồ sơ Uỷ thác cho vay → mở Chi tiết 1 hồ sơ đang ở trạng thái tương ứng.</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>1. Ở CHI TIẾT HỒ SƠ — xác nhận process bar
 2. Chuyển tab THÔNG TIN THẨM ĐỊNH HỒ SƠ
@@ -1774,66 +1774,66 @@
 4. Quay lại CHI TIẾT HỒ SƠ</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Thanh process vẫn đúng trạng thái (không reset / không mất highlight).
 Behavior theo UI: process bar sticky trên các tab hoặc luôn đúng khi quay lại chi tiết — ghi nhận thực tế.</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>NEW — merge vào file gốc, không đụng TC cũ</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Quan_ly_cho_vay</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Quan_ly_cho_vay</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>TC_PROC_011</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Sau khi cập nhật trạng thái (workflow) — process bar highlight bước mới</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Có quyền đẩy trạng thái hồ sơ (tiếp nhận / phân công / thẩm định / ký duyệt) theo luồng hệ thống. [TBD tên action thực tế]</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>1. Mở chi tiết hồ sơ ở trạng thái N
 2. Thực hiện action chuyển sang trạng thái N+1 (theo UI)
 3. Quan sát thanh process</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Highlight chuyển sang bước tương ứng trạng thái mới.
 Bước cũ chuyển style completed.
 List cập nhật cùng trạng thái mới.</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Assumption: có action chuyển trạng thái trên UI</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>
@@ -1858,124 +1858,124 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Sheet "TC mới" nằm ĐẦU FILE — mở file này sẽ thấy ngay</t>
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>QUAN TRỌNG — Merge TC mới vào file gốc</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>File gốc (máy local): C:\Users\hant2\Desktop\HATC\Output\Quan_ly_cho_vay_ fix comment</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Cloud agent KHÔNG đọc được file gốc → xuất sheet TC_MOI (bôi vàng).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Cách merge:</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>1. Mở file gốc Excel (giữ nguyên mọi TC + cột Kết quả test cũ).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2. Copy toàn bộ dòng Flag=NEW từ sheet TC_MOI.</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2. Mở sheet ĐẦU TIÊN tên đúng: "TC mới" (bôi vàng).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>3. Paste vào sheet đầu (Danh sách / Sửa-Xóa) và sheet Chi tiết tương ứng.</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>3. Copy dòng Flag=NEW → paste thêm vào sheet gốc tương ứng (không ghi đè Kết quả test cũ).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>4. KHÔNG ghi đè / xóa TC cũ; KHÔNG sửa cột Kết quả test đã có.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>5. Đổi ID_TC cho khớp sequence file gốc nếu team đánh số liên tục.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>6. Giữ tô vàng các dòng mới để review.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Phạm vi TC mới:</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>- Sửa hồ sơ từ danh sách (sheet đầu) — gồm phần Tài sản đảm bảo</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>- Xóa hồ sơ từ danh sách (sheet đầu)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>- Thanh process trên Chi tiết hồ sơ — highlight theo TRẠNG THÁI HỒ SƠ</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Process steps (UI): Chờ tiếp nhận → Chờ phân công → Chờ thẩm định → Chờ ký duyệt → Đã ký duyệt</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Assumption/TBD: message success/validate nguyên văn; rule Sửa/Xóa theo trạng thái — confirm SRS.</t>
         </is>
@@ -2005,37 +2005,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Khu vực</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Field / Control</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Nguồn UI</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pattern TC</t>
         </is>
@@ -2482,22 +2482,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Est. TC</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Patterns</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
@@ -2572,6 +2572,7 @@
       <c r="B5" t="n">
         <v>26</v>
       </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>User đã yêu cầu update — gen trực tiếp</t>

</xml_diff>